<commit_message>
id3 & mp3 COMM mapping coding exploration
</commit_message>
<xml_diff>
--- a/src/generated_files/MusicBrainz_Picard_Tag_Map.xlsx
+++ b/src/generated_files/MusicBrainz_Picard_Tag_Map.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MusicProcessing\src\generated_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{964A0833-8B8E-44AA-8274-0B85E5AA2E6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEA14D2F-7D74-4506-828C-9C4B7DC0939A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3835,6 +3835,9 @@
       <c r="B94" s="14"/>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H94">
+    <sortCondition ref="A2:A94"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>

</xml_diff>